<commit_message>
Correct Taobao project owner data
</commit_message>
<xml_diff>
--- a/data/数据源8.10-8.14.xlsx
+++ b/data/数据源8.10-8.14.xlsx
@@ -796,6 +796,9 @@
     <t>淘宝闪购</t>
   </si>
   <si>
+    <t>郭周洲</t>
+  </si>
+  <si>
     <t>1-3w</t>
   </si>
   <si>
@@ -1066,9 +1069,6 @@
   </si>
   <si>
     <t>三个月</t>
-  </si>
-  <si>
-    <t>郭周洲</t>
   </si>
   <si>
     <t>全职</t>
@@ -2378,7 +2378,7 @@
   <sheetFormatPr defaultColWidth="9.64285714285714" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="7" width="19" customWidth="1"/>
-    <col min="8" max="8" width="9.64285714285714" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="9.64285714285714" customWidth="1"/>
     <col min="9" max="13" width="19" customWidth="1"/>
     <col min="14" max="14" width="8.71428571428571" customWidth="1"/>
     <col min="15" max="15" width="10.5714285714286" customWidth="1"/>
@@ -4848,7 +4848,7 @@
         <v>163</v>
       </c>
       <c r="D39" t="s">
-        <v>86</v>
+        <v>164</v>
       </c>
       <c r="E39" t="s">
         <v>29</v>
@@ -4857,7 +4857,7 @@
         <v>30</v>
       </c>
       <c r="G39" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I39" t="s">
         <v>32</v>
@@ -4896,16 +4896,16 @@
     </row>
     <row r="40" ht="25.5" customHeight="1" spans="1:22">
       <c r="A40" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B40" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C40" t="s">
         <v>163</v>
       </c>
       <c r="D40" t="s">
-        <v>86</v>
+        <v>164</v>
       </c>
       <c r="E40" t="s">
         <v>29</v>
@@ -4914,7 +4914,7 @@
         <v>30</v>
       </c>
       <c r="G40" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I40" t="s">
         <v>32</v>
@@ -4953,16 +4953,16 @@
     </row>
     <row r="41" ht="25.5" customHeight="1" spans="1:22">
       <c r="A41" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B41" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C41" t="s">
         <v>163</v>
       </c>
       <c r="D41" t="s">
-        <v>86</v>
+        <v>164</v>
       </c>
       <c r="E41" t="s">
         <v>46</v>
@@ -4971,7 +4971,7 @@
         <v>30</v>
       </c>
       <c r="G41" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I41" t="s">
         <v>121</v>
@@ -5010,16 +5010,16 @@
     </row>
     <row r="42" ht="25.5" customHeight="1" spans="1:22">
       <c r="A42" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B42" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C42" t="s">
         <v>163</v>
       </c>
       <c r="D42" t="s">
-        <v>86</v>
+        <v>164</v>
       </c>
       <c r="E42" t="s">
         <v>46</v>
@@ -5028,7 +5028,7 @@
         <v>30</v>
       </c>
       <c r="G42" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I42" t="s">
         <v>121</v>
@@ -5067,16 +5067,16 @@
     </row>
     <row r="43" ht="25.5" customHeight="1" spans="1:22">
       <c r="A43" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B43" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C43" t="s">
         <v>163</v>
       </c>
       <c r="D43" t="s">
-        <v>86</v>
+        <v>164</v>
       </c>
       <c r="E43" t="s">
         <v>29</v>
@@ -5121,10 +5121,10 @@
     </row>
     <row r="44" ht="25.5" customHeight="1" spans="1:22">
       <c r="A44" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B44" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C44" t="s">
         <v>27</v>
@@ -5139,7 +5139,7 @@
         <v>30</v>
       </c>
       <c r="G44" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I44" t="s">
         <v>121</v>
@@ -5178,10 +5178,10 @@
     </row>
     <row r="45" ht="25.5" customHeight="1" spans="1:22">
       <c r="A45" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B45" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C45" t="s">
         <v>27</v>
@@ -5196,7 +5196,7 @@
         <v>30</v>
       </c>
       <c r="G45" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I45" t="s">
         <v>32</v>
@@ -5235,10 +5235,10 @@
     </row>
     <row r="46" ht="25.5" customHeight="1" spans="1:22">
       <c r="A46" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B46" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C46" t="s">
         <v>27</v>
@@ -5253,7 +5253,7 @@
         <v>30</v>
       </c>
       <c r="G46" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I46" t="s">
         <v>32</v>
@@ -5292,10 +5292,10 @@
     </row>
     <row r="47" ht="25.5" customHeight="1" spans="1:22">
       <c r="A47" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B47" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C47" t="s">
         <v>27</v>
@@ -5313,7 +5313,7 @@
         <v>130</v>
       </c>
       <c r="I47" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J47">
         <v>0</v>
@@ -5349,7 +5349,7 @@
     </row>
     <row r="48" ht="25.5" customHeight="1" spans="1:22">
       <c r="A48" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B48" t="s">
         <v>125</v>
@@ -5361,7 +5361,7 @@
         <v>79</v>
       </c>
       <c r="E48" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F48" t="s">
         <v>30</v>
@@ -5409,7 +5409,7 @@
     </row>
     <row r="49" ht="25.5" customHeight="1" spans="1:20">
       <c r="A49" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B49" t="s">
         <v>129</v>
@@ -5466,10 +5466,10 @@
     </row>
     <row r="50" ht="25.5" customHeight="1" spans="1:20">
       <c r="A50" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B50" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C50" t="s">
         <v>27</v>
@@ -5520,7 +5520,7 @@
     </row>
     <row r="51" ht="25.5" customHeight="1" spans="1:20">
       <c r="A51" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C51" t="s">
         <v>27</v>
@@ -5535,7 +5535,7 @@
         <v>30</v>
       </c>
       <c r="G51" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I51" t="s">
         <v>48</v>
@@ -5577,7 +5577,7 @@
     <extLst/>
   </autoFilter>
   <dataValidations count="5">
-    <dataValidation type="list" sqref="D2:D50">
+    <dataValidation type="list" sqref="D2:D39 D40:D43 D44:D50">
       <formula1>"张蓉蓉,吴双双,巢育敏,刘新风,后台"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="H2:H50">
@@ -5595,6 +5595,9 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:Y51" listDataValidation="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -5609,52 +5612,52 @@
   <sheetData>
     <row r="1" ht="13" customHeight="1" spans="1:16">
       <c r="A1" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" ht="25.5" customHeight="1" spans="1:16">
@@ -5665,13 +5668,13 @@
         <v>91</v>
       </c>
       <c r="C2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F2" t="s">
         <v>46</v>
@@ -5680,19 +5683,19 @@
         <v>163</v>
       </c>
       <c r="H2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I2" s="2">
         <v>46251</v>
       </c>
       <c r="J2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K2" t="s">
-        <v>209</v>
+        <v>164</v>
       </c>
       <c r="L2" t="s">
-        <v>209</v>
+        <v>164</v>
       </c>
       <c r="M2" t="s">
         <v>210</v>
@@ -5715,13 +5718,13 @@
         <v>42</v>
       </c>
       <c r="C3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D3" t="s">
         <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F3" t="s">
         <v>29</v>
@@ -5765,13 +5768,13 @@
         <v>74</v>
       </c>
       <c r="C4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D4" t="s">
         <v>218</v>
       </c>
       <c r="E4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F4" t="s">
         <v>46</v>
@@ -5786,7 +5789,7 @@
         <v>46160</v>
       </c>
       <c r="J4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K4" t="s">
         <v>79</v>
@@ -5815,13 +5818,13 @@
         <v>42</v>
       </c>
       <c r="C5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D5" t="s">
         <v>220</v>
       </c>
       <c r="E5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F5" t="s">
         <v>29</v>
@@ -5836,7 +5839,7 @@
         <v>46167</v>
       </c>
       <c r="J5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K5" t="s">
         <v>50</v>
@@ -5865,13 +5868,13 @@
         <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D6" t="s">
         <v>222</v>
       </c>
       <c r="E6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F6" t="s">
         <v>46</v>
@@ -5886,7 +5889,7 @@
         <v>46168</v>
       </c>
       <c r="J6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K6" t="s">
         <v>50</v>
@@ -5915,13 +5918,13 @@
         <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D7" t="s">
         <v>223</v>
       </c>
       <c r="E7" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F7" t="s">
         <v>59</v>
@@ -5936,7 +5939,7 @@
         <v>46174</v>
       </c>
       <c r="J7" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K7" t="s">
         <v>50</v>
@@ -5965,13 +5968,13 @@
         <v>74</v>
       </c>
       <c r="C8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D8" t="s">
         <v>224</v>
       </c>
       <c r="E8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F8" t="s">
         <v>29</v>
@@ -6015,13 +6018,13 @@
         <v>74</v>
       </c>
       <c r="C9" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D9" t="s">
         <v>226</v>
       </c>
       <c r="E9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F9" t="s">
         <v>46</v>
@@ -6036,7 +6039,7 @@
         <v>46161</v>
       </c>
       <c r="J9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K9" t="s">
         <v>79</v>
@@ -6065,13 +6068,13 @@
         <v>74</v>
       </c>
       <c r="C10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D10" t="s">
         <v>228</v>
       </c>
       <c r="E10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F10" t="s">
         <v>46</v>
@@ -6086,7 +6089,7 @@
         <v>46161</v>
       </c>
       <c r="J10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K10" t="s">
         <v>79</v>
@@ -6115,13 +6118,13 @@
         <v>74</v>
       </c>
       <c r="C11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D11" t="s">
         <v>229</v>
       </c>
       <c r="E11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F11" t="s">
         <v>46</v>
@@ -6136,7 +6139,7 @@
         <v>46167</v>
       </c>
       <c r="J11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K11" t="s">
         <v>86</v>
@@ -6165,13 +6168,13 @@
         <v>74</v>
       </c>
       <c r="C12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D12" t="s">
         <v>230</v>
       </c>
       <c r="E12" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F12" t="s">
         <v>46</v>
@@ -6186,7 +6189,7 @@
         <v>46170</v>
       </c>
       <c r="J12" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K12" t="s">
         <v>79</v>
@@ -6215,13 +6218,13 @@
         <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D13" t="s">
         <v>231</v>
       </c>
       <c r="E13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F13" t="s">
         <v>46</v>
@@ -6236,7 +6239,7 @@
         <v>46164</v>
       </c>
       <c r="J13" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K13" t="s">
         <v>86</v>
@@ -6265,13 +6268,13 @@
         <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D14" t="s">
         <v>233</v>
       </c>
       <c r="E14" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F14" t="s">
         <v>46</v>
@@ -6286,7 +6289,7 @@
         <v>46181</v>
       </c>
       <c r="J14" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K14" t="s">
         <v>50</v>
@@ -6315,13 +6318,13 @@
         <v>74</v>
       </c>
       <c r="C15" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D15" t="s">
         <v>234</v>
       </c>
       <c r="E15" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F15" t="s">
         <v>46</v>
@@ -6336,7 +6339,7 @@
         <v>46174</v>
       </c>
       <c r="J15" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K15" t="s">
         <v>86</v>
@@ -6365,13 +6368,13 @@
         <v>74</v>
       </c>
       <c r="C16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D16" t="s">
         <v>236</v>
       </c>
       <c r="E16" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F16" t="s">
         <v>46</v>
@@ -6386,7 +6389,7 @@
         <v>46174</v>
       </c>
       <c r="J16" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K16" t="s">
         <v>86</v>
@@ -6415,13 +6418,13 @@
         <v>42</v>
       </c>
       <c r="C17" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D17" t="s">
         <v>237</v>
       </c>
       <c r="E17" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F17" t="s">
         <v>29</v>
@@ -6436,7 +6439,7 @@
         <v>46181</v>
       </c>
       <c r="J17" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K17" t="s">
         <v>50</v>
@@ -6465,13 +6468,13 @@
         <v>42</v>
       </c>
       <c r="C18" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D18" t="s">
         <v>238</v>
       </c>
       <c r="E18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F18" t="s">
         <v>29</v>
@@ -6486,7 +6489,7 @@
         <v>46188</v>
       </c>
       <c r="J18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K18" t="s">
         <v>50</v>
@@ -6515,13 +6518,13 @@
         <v>42</v>
       </c>
       <c r="C19" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D19" t="s">
         <v>239</v>
       </c>
       <c r="E19" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F19" t="s">
         <v>29</v>
@@ -6536,7 +6539,7 @@
         <v>46188</v>
       </c>
       <c r="J19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K19" t="s">
         <v>50</v>
@@ -6565,13 +6568,13 @@
         <v>42</v>
       </c>
       <c r="C20" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D20" t="s">
         <v>240</v>
       </c>
       <c r="E20" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F20" t="s">
         <v>46</v>
@@ -6586,7 +6589,7 @@
         <v>46188</v>
       </c>
       <c r="J20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K20" t="s">
         <v>50</v>
@@ -6615,13 +6618,13 @@
         <v>42</v>
       </c>
       <c r="C21" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D21" t="s">
         <v>241</v>
       </c>
       <c r="E21" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F21" t="s">
         <v>29</v>
@@ -6636,7 +6639,7 @@
         <v>46188</v>
       </c>
       <c r="J21" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K21" t="s">
         <v>50</v>
@@ -6665,13 +6668,13 @@
         <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D22" t="s">
         <v>242</v>
       </c>
       <c r="E22" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F22" t="s">
         <v>46</v>
@@ -6686,7 +6689,7 @@
         <v>46196</v>
       </c>
       <c r="J22" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K22" t="s">
         <v>93</v>
@@ -6715,13 +6718,13 @@
         <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D23" t="s">
         <v>243</v>
       </c>
       <c r="E23" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F23" t="s">
         <v>46</v>
@@ -6736,7 +6739,7 @@
         <v>46198</v>
       </c>
       <c r="J23" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K23" t="s">
         <v>93</v>
@@ -6765,13 +6768,13 @@
         <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D24" t="s">
         <v>244</v>
       </c>
       <c r="E24" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F24" t="s">
         <v>46</v>
@@ -6786,7 +6789,7 @@
         <v>46199</v>
       </c>
       <c r="J24" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K24" t="s">
         <v>93</v>
@@ -6815,13 +6818,13 @@
         <v>42</v>
       </c>
       <c r="C25" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D25" t="s">
         <v>246</v>
       </c>
       <c r="E25" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F25" t="s">
         <v>46</v>
@@ -6836,7 +6839,7 @@
         <v>46195</v>
       </c>
       <c r="J25" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K25" t="s">
         <v>50</v>
@@ -6915,7 +6918,7 @@
         <v>91</v>
       </c>
       <c r="C27" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D27" t="s">
         <v>254</v>
@@ -6936,7 +6939,7 @@
         <v>46204</v>
       </c>
       <c r="J27" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K27" t="s">
         <v>79</v>
@@ -6965,7 +6968,7 @@
         <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D28" t="s">
         <v>257</v>
@@ -6986,7 +6989,7 @@
         <v>46204</v>
       </c>
       <c r="J28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K28" t="s">
         <v>79</v>
@@ -7265,7 +7268,7 @@
         <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D34" t="s">
         <v>266</v>
@@ -7286,13 +7289,13 @@
         <v>46209</v>
       </c>
       <c r="J34" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K34" t="s">
-        <v>209</v>
+        <v>164</v>
       </c>
       <c r="L34" t="s">
-        <v>209</v>
+        <v>164</v>
       </c>
       <c r="M34" t="s">
         <v>210</v>
@@ -7315,13 +7318,13 @@
         <v>91</v>
       </c>
       <c r="C35" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D35" t="s">
         <v>268</v>
       </c>
       <c r="E35" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F35" t="s">
         <v>46</v>
@@ -7336,7 +7339,7 @@
         <v>46204</v>
       </c>
       <c r="J35" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K35" t="s">
         <v>93</v>
@@ -7415,13 +7418,13 @@
         <v>122</v>
       </c>
       <c r="C37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D37" t="s">
         <v>270</v>
       </c>
       <c r="E37" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F37" t="s">
         <v>46</v>
@@ -7436,7 +7439,7 @@
         <v>46209</v>
       </c>
       <c r="J37" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K37" t="s">
         <v>93</v>
@@ -7465,13 +7468,13 @@
         <v>42</v>
       </c>
       <c r="C38" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D38" t="s">
         <v>272</v>
       </c>
       <c r="E38" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F38" t="s">
         <v>46</v>
@@ -7486,7 +7489,7 @@
         <v>46224</v>
       </c>
       <c r="J38" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K38" t="s">
         <v>79</v>
@@ -7515,7 +7518,7 @@
         <v>42</v>
       </c>
       <c r="C39" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D39" t="s">
         <v>273</v>
@@ -7536,7 +7539,7 @@
         <v>46209</v>
       </c>
       <c r="J39" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K39" t="s">
         <v>79</v>
@@ -7565,7 +7568,7 @@
         <v>42</v>
       </c>
       <c r="C40" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D40" t="s">
         <v>274</v>
@@ -7586,7 +7589,7 @@
         <v>46209</v>
       </c>
       <c r="J40" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K40" t="s">
         <v>79</v>
@@ -7615,7 +7618,7 @@
         <v>116</v>
       </c>
       <c r="C41" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D41" t="s">
         <v>275</v>
@@ -7636,7 +7639,7 @@
         <v>46209</v>
       </c>
       <c r="J41" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K41" t="s">
         <v>79</v>
@@ -7665,13 +7668,13 @@
         <v>122</v>
       </c>
       <c r="C42" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D42" t="s">
         <v>276</v>
       </c>
       <c r="E42" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F42" t="s">
         <v>46</v>
@@ -7686,7 +7689,7 @@
         <v>46210</v>
       </c>
       <c r="J42" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K42" t="s">
         <v>93</v>
@@ -7715,13 +7718,13 @@
         <v>122</v>
       </c>
       <c r="C43" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D43" t="s">
         <v>277</v>
       </c>
       <c r="E43" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F43" t="s">
         <v>46</v>
@@ -7736,7 +7739,7 @@
         <v>46209</v>
       </c>
       <c r="J43" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K43" t="s">
         <v>93</v>
@@ -7815,7 +7818,7 @@
         <v>134</v>
       </c>
       <c r="C45" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D45" t="s">
         <v>281</v>
@@ -7836,7 +7839,7 @@
         <v>46210</v>
       </c>
       <c r="J45" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K45" t="s">
         <v>86</v>
@@ -7865,7 +7868,7 @@
         <v>134</v>
       </c>
       <c r="C46" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D46" t="s">
         <v>283</v>
@@ -7886,7 +7889,7 @@
         <v>46210</v>
       </c>
       <c r="J46" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K46" t="s">
         <v>86</v>
@@ -7915,7 +7918,7 @@
         <v>134</v>
       </c>
       <c r="C47" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D47" t="s">
         <v>284</v>
@@ -7936,7 +7939,7 @@
         <v>46210</v>
       </c>
       <c r="J47" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K47" t="s">
         <v>86</v>
@@ -7965,7 +7968,7 @@
         <v>134</v>
       </c>
       <c r="C48" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D48" t="s">
         <v>285</v>
@@ -7986,7 +7989,7 @@
         <v>46210</v>
       </c>
       <c r="J48" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K48" t="s">
         <v>86</v>
@@ -8259,13 +8262,13 @@
         <v>122</v>
       </c>
       <c r="C54" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D54" t="s">
         <v>291</v>
       </c>
       <c r="E54" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F54" t="s">
         <v>46</v>
@@ -8280,7 +8283,7 @@
         <v>46217</v>
       </c>
       <c r="J54" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K54" t="s">
         <v>93</v>
@@ -8309,13 +8312,13 @@
         <v>122</v>
       </c>
       <c r="C55" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D55" t="s">
         <v>292</v>
       </c>
       <c r="E55" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F55" t="s">
         <v>46</v>
@@ -8330,7 +8333,7 @@
         <v>46223</v>
       </c>
       <c r="J55" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K55" t="s">
         <v>93</v>
@@ -8359,13 +8362,13 @@
         <v>122</v>
       </c>
       <c r="C56" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D56" t="s">
         <v>293</v>
       </c>
       <c r="E56" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F56" t="s">
         <v>46</v>
@@ -8380,7 +8383,7 @@
         <v>46217</v>
       </c>
       <c r="J56" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K56" t="s">
         <v>93</v>
@@ -8409,13 +8412,13 @@
         <v>122</v>
       </c>
       <c r="C57" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D57" t="s">
         <v>294</v>
       </c>
       <c r="E57" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F57" t="s">
         <v>46</v>
@@ -8430,7 +8433,7 @@
         <v>46217</v>
       </c>
       <c r="J57" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K57" t="s">
         <v>93</v>
@@ -8459,13 +8462,13 @@
         <v>122</v>
       </c>
       <c r="C58" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D58" t="s">
         <v>295</v>
       </c>
       <c r="E58" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F58" t="s">
         <v>46</v>
@@ -8509,7 +8512,7 @@
         <v>134</v>
       </c>
       <c r="C59" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D59" t="s">
         <v>298</v>
@@ -8530,7 +8533,7 @@
         <v>46216</v>
       </c>
       <c r="J59" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K59" t="s">
         <v>224</v>
@@ -8707,13 +8710,13 @@
         <v>122</v>
       </c>
       <c r="C63" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D63" t="s">
         <v>304</v>
       </c>
       <c r="E63" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F63" t="s">
         <v>46</v>
@@ -8728,7 +8731,7 @@
         <v>46223</v>
       </c>
       <c r="J63" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K63" t="s">
         <v>93</v>
@@ -8757,13 +8760,13 @@
         <v>122</v>
       </c>
       <c r="C64" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D64" t="s">
         <v>305</v>
       </c>
       <c r="E64" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F64" t="s">
         <v>46</v>
@@ -8778,7 +8781,7 @@
         <v>46224</v>
       </c>
       <c r="J64" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K64" t="s">
         <v>93</v>
@@ -8878,7 +8881,7 @@
         <v>46220</v>
       </c>
       <c r="J66" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K66" t="s">
         <v>79</v>
@@ -8928,7 +8931,7 @@
         <v>46220</v>
       </c>
       <c r="J67" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K67" t="s">
         <v>79</v>
@@ -8978,7 +8981,7 @@
         <v>46220</v>
       </c>
       <c r="J68" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K68" t="s">
         <v>79</v>
@@ -9157,7 +9160,7 @@
         <v>134</v>
       </c>
       <c r="C72" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D72" t="s">
         <v>316</v>
@@ -9178,7 +9181,7 @@
         <v>46224</v>
       </c>
       <c r="J72" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K72" t="s">
         <v>86</v>
@@ -9207,7 +9210,7 @@
         <v>134</v>
       </c>
       <c r="C73" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D73" t="s">
         <v>317</v>
@@ -9228,7 +9231,7 @@
         <v>46224</v>
       </c>
       <c r="J73" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K73" t="s">
         <v>86</v>
@@ -9403,13 +9406,13 @@
         <v>122</v>
       </c>
       <c r="C77" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D77" t="s">
         <v>321</v>
       </c>
       <c r="E77" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F77" t="s">
         <v>46</v>
@@ -9424,7 +9427,7 @@
         <v>46232</v>
       </c>
       <c r="J77" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K77" t="s">
         <v>86</v>
@@ -9453,7 +9456,7 @@
         <v>134</v>
       </c>
       <c r="C78" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D78" t="s">
         <v>322</v>
@@ -9474,7 +9477,7 @@
         <v>46230</v>
       </c>
       <c r="J78" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K78" t="s">
         <v>224</v>
@@ -9503,7 +9506,7 @@
         <v>134</v>
       </c>
       <c r="C79" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D79" t="s">
         <v>323</v>
@@ -9524,7 +9527,7 @@
         <v>46230</v>
       </c>
       <c r="J79" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K79" t="s">
         <v>224</v>

</xml_diff>